<commit_message>
Corrige importacion de la plantilla Diagnostico Social V4
- Lector por celda exacta: la cabecera ya no toma el rotulo vecino como
  valor y F-DS-01 reconoce el codigo de bloque.
- Importa todos los campos de F-DS-01..07: textos, casillas «X»,
  desplegables y codigos de la hoja _Codigos (GL, A, F, SH, LT, 2...).
- Una plantilla en blanco ya no se reporta como 7 fichas con datos.
- Avisos por bloque inexistente, fecha fuera de rango y coordenadas UTM
  fuera del ambito 17S.
- El mensaje de autocompletado persiste tras el rerun; la precarga de
  datos generales no se borra al cambiar de bloque.
- Plantilla: desplegables Estado/Antig. de F-DS-05 movidos a F/G
  (estaban ocultos en la celda combinada C:E); rotulo Papelografos en
  F-DS-04.
- Listas de opciones de F-DS-03/04/05/07 centralizadas en fds_listas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NosAPHBSnVBDB8qxbDWoFC
</commit_message>
<xml_diff>
--- a/Plantilla_Diagnostico_Social_IN_Piura_V4.xlsx
+++ b/Plantilla_Diagnostico_Social_IN_Piura_V4.xlsx
@@ -17808,8 +17808,10 @@
     </row>
     <row r="25" spans="1:14" s="48" customFormat="1" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="65"/>
-      <c r="B25" s="321" t="s">
-        <v>393</v>
+      <c r="B25" s="321" t="inlineStr">
+        <is>
+          <t>Papelógrafos</t>
+        </is>
       </c>
       <c r="C25" s="118"/>
       <c r="D25" s="118"/>
@@ -20524,13 +20526,13 @@
           <x14:formula1>
             <xm:f>_Listas!$Y$2:$Y$6</xm:f>
           </x14:formula1>
-          <xm:sqref>D14 D15 D16 D17 D18 D19 D20 D21</xm:sqref>
+          <xm:sqref>F14 F15 F16 F17 F18 F19 F20 F21</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0500-000002000000}">
           <x14:formula1>
             <xm:f>_Listas!$Z$2:$Z$7</xm:f>
           </x14:formula1>
-          <xm:sqref>E14 E15 E16 E17 E18 E19 E20 E21</xm:sqref>
+          <xm:sqref>G14 G15 G16 G17 G18 G19 G20 G21</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>